<commit_message>
Implemented Place Order with Payment test using DataProvider and POM
</commit_message>
<xml_diff>
--- a/src/main/resources/TestData/TestData.xlsx
+++ b/src/main/resources/TestData/TestData.xlsx
@@ -5,11 +5,12 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="ValidLogin" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="InvalidLogin" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="PlaceOrderData" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -21,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="13">
   <si>
     <t xml:space="preserve">Email</t>
   </si>
@@ -39,6 +40,27 @@
   </si>
   <si>
     <t xml:space="preserve">And@123</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Card</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CVC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Month</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Year</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Anurag Pandey</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4111111111156</t>
   </si>
 </sst>
 </file>
@@ -78,8 +100,8 @@
       <charset val="1"/>
     </font>
     <font>
-      <sz val="10"/>
-      <color rgb="FF0000FF"/>
+      <b val="true"/>
+      <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
@@ -127,7 +149,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -140,8 +162,12 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -313,18 +339,18 @@
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="2" t="s">
         <v>5</v>
       </c>
     </row>
@@ -341,4 +367,78 @@
     <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:G2"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="38.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="25.74"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="36.17"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E2" s="1" t="n">
+        <v>815</v>
+      </c>
+      <c r="F2" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="G2" s="1" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A2" r:id="rId1" display="anuragpandey930565@gmail.com"/>
+    <hyperlink ref="B2" r:id="rId2" display="Anurag@123"/>
+  </hyperlinks>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Implemented Contact Us automation using POM and DataProvider
</commit_message>
<xml_diff>
--- a/src/main/resources/TestData/TestData.xlsx
+++ b/src/main/resources/TestData/TestData.xlsx
@@ -5,12 +5,13 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="ValidLogin" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="InvalidLogin" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="PlaceOrderData" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="ContactUS" sheetId="4" state="visible" r:id="rId6"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -22,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="19">
   <si>
     <t xml:space="preserve">Email</t>
   </si>
@@ -61,6 +62,24 @@
   </si>
   <si>
     <t xml:space="preserve">4111111111156</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NAME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EMAIL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SUBJECT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MESSAGE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FeedBack</t>
+  </si>
+  <si>
+    <t xml:space="preserve">This is the Test</t>
   </si>
 </sst>
 </file>
@@ -441,4 +460,57 @@
     <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="18.64"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="34.92"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="16.69"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="22.68"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="B1" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="C1" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="D1" s="0" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="0" t="s">
+        <v>11</v>
+      </c>
+      <c r="B2" s="0" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" s="0" t="s">
+        <v>17</v>
+      </c>
+      <c r="D2" s="0" t="s">
+        <v>18</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add subscription test cases for home and cart pages
</commit_message>
<xml_diff>
--- a/src/main/resources/TestData/TestData.xlsx
+++ b/src/main/resources/TestData/TestData.xlsx
@@ -5,13 +5,14 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="ValidLogin" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="InvalidLogin" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="PlaceOrderData" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="ContactUS" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="Subscription" sheetId="5" state="visible" r:id="rId7"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -23,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="20">
   <si>
     <t xml:space="preserve">Email</t>
   </si>
@@ -80,6 +81,9 @@
   </si>
   <si>
     <t xml:space="preserve">This is the Test</t>
+  </si>
+  <si>
+    <t xml:space="preserve">anuragpandey@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -89,7 +93,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -121,6 +125,13 @@
     <font>
       <b val="true"/>
       <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF0000FF"/>
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
@@ -168,7 +179,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -187,6 +198,10 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -470,37 +485,37 @@
   <dimension ref="A1:D2"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="18.64"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="34.92"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="16.69"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="22.68"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="18.64"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="34.92"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="16.69"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="22.68"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" s="1" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+      <c r="A2" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="D2" s="0" t="s">
+      <c r="D2" s="1" t="s">
         <v>18</v>
       </c>
     </row>
@@ -513,4 +528,36 @@
     <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:A2"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="0" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="5" t="s">
+        <v>19</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A2" r:id="rId1" display="anuragpandey@gmail.com"/>
+  </hyperlinks>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add product review test with success message validation
</commit_message>
<xml_diff>
--- a/src/main/resources/TestData/TestData.xlsx
+++ b/src/main/resources/TestData/TestData.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="4"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="ValidLogin" sheetId="1" state="visible" r:id="rId3"/>
@@ -13,6 +13,7 @@
     <sheet name="PlaceOrderData" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="ContactUS" sheetId="4" state="visible" r:id="rId6"/>
     <sheet name="Subscription" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="ProductReview" sheetId="6" state="visible" r:id="rId8"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -24,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="23">
   <si>
     <t xml:space="preserve">Email</t>
   </si>
@@ -84,6 +85,15 @@
   </si>
   <si>
     <t xml:space="preserve">anuragpandey@gmail.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Message </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Anurag</t>
+  </si>
+  <si>
+    <t xml:space="preserve">I love you </t>
   </si>
 </sst>
 </file>
@@ -537,6 +547,9 @@
   </sheetPr>
   <dimension ref="A1:A2"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="47.86"/>
+  </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="0" t="s">
@@ -560,4 +573,58 @@
     <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="29.25"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1" s="0" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" s="0" t="s">
+        <v>21</v>
+      </c>
+      <c r="D2" s="0" t="s">
+        <v>22</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A2" r:id="rId1" display="anuragpandey930565@gmail.com"/>
+    <hyperlink ref="B2" r:id="rId2" display="Anurag@123"/>
+  </hyperlinks>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>